<commit_message>
compute optimised logic changes
</commit_message>
<xml_diff>
--- a/output_results.xlsx
+++ b/output_results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -501,7 +501,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Free: Debian, CentOS, CoreOS, Ubuntu or BYOL</t>
+          <t>Paid: Windows Server</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -514,47 +514,47 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>e2-micro</t>
+          <t>e2-standard-2</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://cloud.google.com/products/calculator?dl=CjhDaVEzTTJVM1lqQTNOUzFqWmprekxUUmhZall0WWpFM05TMWpNbVZpTVRkbVlUSXdObVFRQVE9PRAIGiQ2M0RDQzk4My02RjBCLTQ1RDMtQUI4NS0xRkFEMERFNDI1RTI</t>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVEwTlRGalpHRm1aQzFpWVdVM0xUUmtNRGt0WW1NME5TMDJPVGsyWW1ZMk5HVTNORGtRQVE9PRAIGiQ0Rjg4NzgxRS0xRTQyLTQyMzItQkVDOC0zQUNDRDdGMUQyQUI</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>$5.38</t>
+          <t>$215.74</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://cloud.google.com/products/calculator?dl=CjhDaVEzTTJVM1lqQTNOUzFqWmprekxUUmhZall0WWpFM05TMWpNbVZpTVRkbVlUSXdObVFRQVE9PRAIGiQ2M0RDQzk4My02RjBCLTQ1RDMtQUI4NS0xRkFEMERFNDI1RTI</t>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVF5WVRJNE56QmlZaTB6TWpabExUUmtZamt0T0RnNU55MHhOR1kxTkRKa1pUaGhOMlVRQVE9PRAIGiREODY4RERBQy0zNUZFLTRBMjMtQjdCRS02NUQxMTc5MENFNjQ</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>$5.38</t>
+          <t>$199.27</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>https://cloud.google.com/products/calculator?dl=CjhDaVEzTTJVM1lqQTNOUzFqWmprekxUUmhZall0WWpFM05TMWpNbVZpTVRkbVlUSXdObVFRQVE9PRAIGiQ2M0RDQzk4My02RjBCLTQ1RDMtQUI4NS0xRkFEMERFNDI1RTI</t>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJpTURrNE1qUmlZUzB5TkRZeExUUTBNak10WWpObVppMW1PV1JoT1RZd056TmxaalVRQVE9PRAIGiQxMkE0NUNCRi1DOUI1LTRFMEYtQkQ2QS0zQUIzNzk1RDIwODQ</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>$5.38</t>
+          <t>$185.62</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>https://cloud.google.com/products/calculator?dl=CjhDaVEzTTJVM1lqQTNOUzFqWmprekxUUmhZall0WWpFM05TMWpNbVZpTVRkbVlUSXdObVFRQVE9PRAIGiQ2M0RDQzk4My02RjBCLTQ1RDMtQUI4NS0xRkFEMERFNDI1RTI</t>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVEyTnpWa1l6Sm1aUzFpT0dJMExUUTNOVE10T1dFMk1TMHlOR1poWldWbU1tTmxabUlRQVE9PRAIGiRDNDY0OUMxMS05MkJGLTQyMjktODM5Ni0wNTg2NTkxM0ZBM0M</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>$5.38</t>
+          <t>$170.96</t>
         </is>
       </c>
     </row>
@@ -564,7 +564,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Free: Debian, CentOS, CoreOS, Ubuntu or BYOL</t>
+          <t>Paid: Windows Server</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -577,47 +577,47 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>e2-small</t>
+          <t>e2-standard-2</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJoTmpNd05XTTJZUzAzTlRNeExUUmtOakF0WWpobE5DMWtZak16TWpkaE5qbGtaVGdRQVE9PRAIGiRBNDEyRkM0OC01NkMwLTRGMzQtOTY2OS1GRDU3M0JGQzZGRTY</t>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJqTldKak9ETm1ZeTAzWWpCakxUUmhZemN0WVRJd1pDMWpZamcwT1RFek4yVmlZeklRQVE9PRAIGiRFOUMyMkIzQy05NjUxLTQ1OEMtOTUxRS04RjQxRTkzQUYzMUE</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>$14.19</t>
+          <t>$215.74</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJoTmpNd05XTTJZUzAzTlRNeExUUmtOakF0WWpobE5DMWtZak16TWpkaE5qbGtaVGdRQVE9PRAIGiRBNDEyRkM0OC01NkMwLTRGMzQtOTY2OS1GRDU3M0JGQzZGRTY</t>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJpWlRRMk5HVTBOeTFqTVRRMkxUUTRZakF0T0dJeE9DMHlNMkUzWVRRM05tWXpZemtRQVE9PRAIGiQ4MDE5QzVBNC1GODY5LTQ4QTQtOTVGQy1FN0NDOTcwNTQyQjE</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>$14.19</t>
+          <t>$199.27</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJoTmpNd05XTTJZUzAzTlRNeExUUmtOakF0WWpobE5DMWtZak16TWpkaE5qbGtaVGdRQVE9PRAIGiRBNDEyRkM0OC01NkMwLTRGMzQtOTY2OS1GRDU3M0JGQzZGRTY</t>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJqT1RkbVlqTmxNeTFoTkRFMUxUUTJNRFl0T0RkbU15MDBNbVZoT0RVNE1UUXhZbVlRQVE9PRAIGiRFREFDN0I1Ni04RDQ3LTQwOTAtQUIxNC0xODY4OUIzN0NBNEM</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>$14.19</t>
+          <t>$185.62</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJoTmpNd05XTTJZUzAzTlRNeExUUmtOakF0WWpobE5DMWtZak16TWpkaE5qbGtaVGdRQVE9PRAIGiRBNDEyRkM0OC01NkMwLTRGMzQtOTY2OS1GRDU3M0JGQzZGRTY</t>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVExT0dOaVpXWTFZeTAwWTJWa0xUUTNaREF0T1dOaU9TMHpaVGhrT0dJMU16Y3pZV01RQVE9PRAIGiQ3RDY4NDEyNi01MzQyLTQ4NTItODVBRS05NjY3QUI1QUM3RUE</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>$14.19</t>
+          <t>$170.96</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Paid: Red Hat Enterprise Linux</t>
+          <t>Free: Debian, CentOS, CoreOS, Ubuntu or BYOL</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -640,47 +640,488 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>e2-small</t>
+          <t>e2-highmem-2</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJsWXpNNU9EWXlNeTA1TW1OaUxUUTNOMk10T0RGaE1TMHhOak0wTjJNMk5qTmtPREVRQVE9PRAIGiRDNDAyRERCMS1ERTA0LTRGODYtOTAyRi1GNjMyMTRCM0YyRkI</t>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVF5TVRZNE0yWTBNeTFqTWpBMkxUUm1NMk10T1dJMU1TMDRNekpsWkRkak1tUmhNVGdRQVE9PRAIGiQyQ0M2QkU3NC1BNjQ5LTQ2M0EtODUzQi03NTkyNjkyNTlFOEE</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>$16.16</t>
+          <t>$219.67</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJsWXpNNU9EWXlNeTA1TW1OaUxUUTNOMk10T0RGaE1TMHhOak0wTjJNMk5qTmtPREVRQVE9PRAIGiRDNDAyRERCMS1ERTA0LTRGODYtOTAyRi1GNjMyMTRCM0YyRkI</t>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVF3T1RkbFlqRmlNeTFqWm1Rd0xUUXlObU10T0dZd05pMWlPR00yT0RnNU5qSXhaVE1RQVE9PRAIGiRDMEUyNjE5NS1CNTNELTQ5QTAtOTc0NC00QUJCM0FBREY0Mzk</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>$16.16</t>
+          <t>$175.23</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJsWXpNNU9EWXlNeTA1TW1OaUxUUTNOMk10T0RGaE1TMHhOak0wTjJNMk5qTmtPREVRQVE9PRAIGiRDNDAyRERCMS1ERTA0LTRGODYtOTAyRi1GNjMyMTRCM0YyRkI</t>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJoWlRnell6RTFOQzB3TWpjMkxUUmpOVEV0WW1ZNU1pMHhZMkUzTm1JME1HSm1NRGNRQVE9PRAIGiQxMEQ3QTZBQi01MTFCLTRGQTgtQjVDNC1GOEFERTVFQTU1MkQ</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>$16.16</t>
+          <t>$138.40</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJsWXpNNU9EWXlNeTA1TW1OaUxUUTNOMk10T0RGaE1TMHhOak0wTjJNMk5qTmtPREVRQVE9PRAIGiRDNDAyRERCMS1ERTA0LTRGODYtOTAyRi1GNjMyMTRCM0YyRkI</t>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVEwTVRrM04yTTNaaTFoTldOakxUUXpNMlF0WVdFeE1TMW1ZVE16WWpKak1tUTJNek1RQVE9PRAIGiRENjE1NDE3Ri02ODI2LTQ4NEEtQjU2OS0yRUIzNDVGNkNFNkQ</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>$16.16</t>
+          <t>$98.86</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Free: Debian, CentOS, CoreOS, Ubuntu or BYOL</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>general purpose</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>e2-highmem-2</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJsTkRnd05XVmxaQzB6T1dFM0xUUXlOR0V0T1RRd1pTMDNOV0kyWVRabVpqTTNOekFRQVE9PRAIGiQyQkQyMkFBNC0yRTE4LTQ2ODAtQTgzQy03RTZDMjY1NzQ3OUY</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>$219.67</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJqWXpaa04yTTFPUzB3WkRNNUxUUXhNR1F0T0Raa09DMW1PVEUwT0dJd05qZGxPRGdRQVE9PRAIGiQwMTI4MjVEQy1EQTMwLTQwQTEtOTUyOS03MkVGRkEwQzU1N0E</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>$175.23</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVEwTmpabFlUY3hZeTB5TnpVeExUUTBOMkl0WVRBek55MHlNRGxsWkdSbE16RTFNVGNRQVE9PRAIGiRCQzA0RkJEQi0wMDZBLTQ4MjAtOTA2OS1BRkJDNzk0QTYzRDA</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>$138.40</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVF5WXpnNE5HRXlPUzA0T0dSbUxUUXlOMk10WVRFek5pMHhPVGN4TUdZMllqRTJNMllRQVE9PRAIGiQ3NEFCNzI4Ni1DNUEwLTQyNkItQjdCNS05NEVBNzk5MDEyRkY</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>$98.86</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Paid: Red Hat Enterprise Linux</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>general purpose</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>e2-standard-2</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJpTTJFMU5UWTBOQzB5T1RreUxUUXlZMkV0WWpBeE5DMHhPRE13TVRSaVpHRXlORGdRQVE9PRAIGiRBM0JDNjhCQS1GREQzLTQ5RTUtQTQxRC03ODU2MEJGQkYzQjI</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>$212.35</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJoTW1aaE1EQXlOQzAyTm1VeExUUm1aR010T0RBeE9DMW1ObVUyWWpGak5qTmtPV0VRQVE9PRAIGiQ4MjFCODQ3Qy1GNjEyLTQxQjgtQkMwNC1ENzEyOUI0MUQyMjc</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>$177.90</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJtWlRGaU0yTmlNQzA1WVRJMUxUUTJZMll0WWpGa01pMHlOREV3Wm1ReVlUSXpaR0lRQVE9PRAIGiQxNjE3MzU1Ni1BMUE0LTRDMzEtODY5Qy1CMTk1RDQ5RTdENjg</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>$149.32</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVF4WWpJMVpHTTNPQzAzWWpVNUxUUm1aRE10WVRGbE5DMHlZVE13TVdJek56a3dZbUlRQVE9PRAIGiQ4RDk0MDczOC00MTBDLTQ3MkEtQjI5OC0zQzI5NTUwNEUyNzg</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>$118.68</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Paid: Windows Server</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>general purpose</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>e2-highmem-2</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVF5T0RVMk1EUTBOeTAyTW1Vd0xUUmlOekF0T0RNMFppMWxaRFkzWmpnNFlXRXlNalVRQVE9PRAIGiRGOEI1NTQxRi05NkRDLTRCRDMtQTA2Ni0zM0EyMjY1MjJEQ0E</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>$364.05</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVE1T0RZM09EVXdaUzFoWkdZNExUUTVPVGd0WWpSaE55MWxNMlUyTkRSaVpHSmhaR1lRQVE9PRAIGiQzMjE2QkQzNS1BQTc1LTRBNTItQkI1QS0yMDRFMTc0NDRGNEE</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>$317.57</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVE1WmpZMU1HWTFaaTFqWlRGbExUUXdNV0V0WW1JellpMDVaVEJrWXpRNE9EazJNelFRQVE9PRAIGiREODY4RjA2OC0xRDFCLTQ4RTItQjZEQi0yNjVBMUEzRTFDQjc</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>$279.03</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVE0TnpSaU4yVmhNaTAxTlRFMUxUUmxabUl0T1RSa05pMW1ZelZsTlRGaU1XUXpZVFFRQVE9PRAIGiRBOTRBREY3OS1CQzZFLTQ5MzYtQTFCMC0zQjA2RjczMTQxNjE</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>$237.70</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Free: Debian, CentOS, CoreOS, Ubuntu or BYOL</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>general purpose</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>e2-highmem-2</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJoWlRSa01ERTVZeTFoTkRJeUxUUmhPV1F0WW1abVlpMW1Nell6TVRVNFlXVTVOR1FRQVE9PRAIGiQ0ODQ2NDVBMy05MzRFLTQ4MkItQkU3Ri0wRDY4OEY2RTU3QzU</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>$229.73</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJoTVRWbVl6ZGlOeTFrWkRCbUxUUTRZVFF0WVdKaE5TMHhPV0ZsT1RGaFpqWXlOVGtRQVE9PRAIGiQwMzdDQTUyMS05QkFFLTRCQTEtODkzMi0xRDJBREVENDNBODU</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>$183.25</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJqWkRNMU9URmpaUzB4WlRZeUxUUTBZemt0T0RRM01pMHhNakZoTlRrNU9ETTFORGtRQVE9PRAIGiRCNTkxMkE3Ni05NUQ3LTQwQzQtQjM0Qy1FQ0I2OTA2QTA3MzM</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>$144.71</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVF5T1RnMlkyUTBNUzFsTXpSa0xUUXhOVGN0T0dWaVlpMWpaRFU1T1dSbVpqZG1ZMllRQVE9PRAIGiREQUZCMzk1OC0xMkJGLTQ5NDEtQTgyRi1EQjY3OERBNDZCQkU</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>$103.38</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Free: Debian, CentOS, CoreOS, Ubuntu or BYOL</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>general purpose</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>e2-highmem-2</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJpWWpjd1lqQTRZUzAzWVdZd0xUUXlNVE10T0Roa01pMDVNamRqWVRnM05UYzNNRFFRQVE9PRAIGiQ4MURDRDdGMC1BMUY2LTRFMzktODM1RC1DRjVGNDdDQkE0RkM</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>$1,837.82</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJqT0RZek5XRXhPUzFtTlRsaExUUTVNRGd0WVdSak5DMDRZall3TWpVellXVmlaVEFRQVE9PRAIGiQ1M0JDRDA0NC1EM0Y1LTREMkUtQTkyQy03NEJFNUExRURFMUQ</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>$1,466.03</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJtTVdRNE9XUTFaaTB5WWpVMExUUm1NVE10WW1JeVpTMDVaVE0yTmpWbU5EY3hOR1lRQVE9PRAIGiQzRTdGQUNENi01NkY0LTRCM0MtODRDMi1CQkVBMThFNzk2NUU</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>$1,157.67</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVE0T1dJMlpESmxaaTAxT1dJMkxUUXdNVE10T0dZMk1pMDVPR1F5TURka1lXSTNNakVRQVE9PRAIGiQyRTZDMjdBRS0wMzg0LTRCOTEtQkQ5Ri00QjVGNDQyNzk3NTA</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>$827.06</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Free: Debian, CentOS, CoreOS, Ubuntu or BYOL</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>general purpose</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>e2-highmem-2</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJpWmpZMU5HUXhaUzA0TVRWaUxUUTNaV1V0T1dVd055MHdOV0ZrTVRJNE16YzJZVE1RQVE9PRAIGiRCNUI1Qjk2NS0yOTFELTQ1OTgtOUQzQi01RUZEODI2MjkyMTg</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>$229.73</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVF6TVRJNU1EWXpOeTB4T1dVMUxUUmpaR0V0T1RBMU15MWtOVFV5TURWaU56UmhNeklRQVE9PRAIGiQ4OUZFODgzNS03RkE1LTREMUQtQjM3My05REY5ODMzQURBRTE</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>$183.25</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVEyWTJRNVpHTTNaaTA1WkRNMkxUUXhaamd0T1dGaU15MDNaamczTVRVNU9HRmtaVFVRQVE9PRAIGiRBMjBCQjcxMy05MzdELTRFQzEtOTgwOS05RkU3QUNEM0Q1REY</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>$144.71</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVEyWVRJMU5EWTBOUzAyWkRJeUxUUmlNMkV0T1dJek9TMHhPVEl5TVdGaU4yVTBaallRQVE9PRAIGiQ0QUFFODVGRS02NzM5LTRCMTUtQjUxQS0yRjI3MjZFOUM0Mjc</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>$103.38</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Free: Debian, CentOS, CoreOS, Ubuntu or BYOL</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>general purpose</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>e2-highmem-2</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVF6TVRBMU5qSTRZaTAxWTJSaExUUTBOamt0WWpJNFpTMDRZemc1T1dNeVlUWmhaV01RQVE9PRAIGiQ4RUU3ODhBOS03OTAxLTQ3REItOTU4QS1BNzEyRDk4NTJENjI</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>$918.91</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVF4WWpVM05UZzRNeTFoT0dabUxUUTFZbUV0WVdKalppMDNPRGc1T0dWa05tWTBaalFRQVE9PRAIGiQ3QkNERDAwMC1EQThGLTQwQzktQUUxMS00Njg4RkIwMDNFNTI</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>$733.02</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVJrTUdRek5tUTVZeTA0TVdJNExUUmxOek10T0RFeE9DMWpNR001WmpsbE5UaGlPRFVRQVE9PRAIGiRBRUYyM0E3QS0xQzU5LTQxMUItOTdENS1GODlEMUQzNEQ5MjQ</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>$578.84</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>https://cloud.google.com/products/calculator?dl=CjhDaVE0TUdRMVlqZzNNaTB5WVdVMExUUmlNMkV0WWpRMllpMDRORGhtWW1RM1pqRmhObU1RQVE9PRAIGiQyMjVFNjNFQi1GNEZFLTRBODctQkYzNy0zNTU0RjE0MDhERTk</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>$413.53</t>
         </is>
       </c>
     </row>

</xml_diff>